<commit_message>
Updated master data and KPI json file for HR vertical
</commit_message>
<xml_diff>
--- a/data/master_data.xlsx
+++ b/data/master_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mishra Ishu Kumar\Downloads\kpi-selector-fullstack\kpi-selector-fullstack\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A83D21F1-CD67-46D7-83E0-EBCE31540535}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6470C9B6-325F-430A-80BB-293380D5BFAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,9 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$970</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$978</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -4881,7 +4881,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4894,6 +4894,18 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -4942,20 +4954,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5265,19 +5290,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>1607</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>698</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -5286,7 +5311,7 @@
       <c r="G1" s="1" t="s">
         <v>1608</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>1609</v>
       </c>
     </row>
@@ -30701,6 +30726,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="40c06f83-eb3a-4154-b6df-c050a871a9a7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d4a8732a-aacb-45a8-aed5-6309649c2e20">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010068AA247FB109614B9C824E32EE240D1D" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f62d1a1f3e04d7282013043d338714c3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d4a8732a-aacb-45a8-aed5-6309649c2e20" xmlns:ns3="40c06f83-eb3a-4154-b6df-c050a871a9a7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="edb964f0ac61e74035de9f95ccc9459a" ns2:_="" ns3:_="">
     <xsd:import namespace="d4a8732a-aacb-45a8-aed5-6309649c2e20"/>
@@ -30913,27 +30958,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0F1D70-8AD9-4EA4-B492-E4F52E050418}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="40c06f83-eb3a-4154-b6df-c050a871a9a7"/>
+    <ds:schemaRef ds:uri="d4a8732a-aacb-45a8-aed5-6309649c2e20"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="40c06f83-eb3a-4154-b6df-c050a871a9a7" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d4a8732a-aacb-45a8-aed5-6309649c2e20">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B43E3947-DC1B-44DF-B577-C2938D9BD05A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B0C6850-3EAD-4D3D-BC46-78E300309E6C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -30950,23 +30994,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B43E3947-DC1B-44DF-B577-C2938D9BD05A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB0F1D70-8AD9-4EA4-B492-E4F52E050418}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="40c06f83-eb3a-4154-b6df-c050a871a9a7"/>
-    <ds:schemaRef ds:uri="d4a8732a-aacb-45a8-aed5-6309649c2e20"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>